<commit_message>
docs(pricing): lock commercial console §6.4 and refresh L3a/L3b artifacts
Document Admin 商务价格 package flow and eng backlog S-01～S-04; update rebuild/outward scripts, quote workbooks, and supply-route input. Exclude local usage export with customer request IDs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-outward-quote-standard.xlsx
+++ b/pricing/output/trinity-outward-quote-standard.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="00_说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="01_标准档报价" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="99_对内索引_勿外发" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_标准档报价" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_对内索引_勿外发" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>缓存命中列；上游成本折/线路/中转站/GM</t>
+          <t>上游成本折/线路/中转站/GM；阶梯列不含缓存（缓存仅目录价列）</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>L2 线上刊例 · trinity-pricing-text.xlsx「线上刊例」USD</t>
+          <t>L2 线上刊例 · trinity-pricing-text.xlsx「线上刊例」USD（入/出/缓）</t>
         </is>
       </c>
     </row>
@@ -650,101 +650,113 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>商务洽谈折扣总表 01（对客折）× 02 推荐成本折（交叉模型）或 01 模型归属</t>
+          <t>定价方案-v0 公开定折矩阵（0.65/0.70/0.75 + 0.78浅折 + Claude 对齐）；模型→成本族取自商务表 01/02；1.0/未映射对外写原价；不抄 L3b 商务深折</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>达档口径</t>
+          <t>公开定折摘要</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>与商务表一致：企业户月消耗按目录价累计（非预存余额）</t>
+          <t>0.65: 8.8/8.5/8.2/7.6/7.2；0.70: 9.0/8.8/8.5/8.0/7.8；0.75: 9.2/9.0/8.7/8.5/8.2；0.78浅折: 9.6/9.4/9.2/8.8/8.5；Claude(非1.0): 9.8/9.5/9.2/9.0/8.8；1.0/未映射: 原价</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>生成日期</t>
+          <t>达档口径</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>与商务表一致：企业户月消耗按目录价累计（非预存余额）</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>有效期（初版暂定）</t>
+          <t>生成日期</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>至 2026-08-31 24:00；过期请向运营索取新版</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>单位</t>
+          <t>有效期（初版暂定）</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>USD / 百万 tokens</t>
+          <t>至 2026-08-31 24:00；过期请向运营索取新版</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>商务表</t>
+          <t>单位</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>保持独立、仅对内；本文件为新建外发表，不覆盖商务表</t>
+          <t>USD / 百万 tokens</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>状态</t>
+          <t>商务表</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>初版草稿 · 待产品/商务确认后正式外发</t>
+          <t>保持独立、仅对内；本文件为新建外发表，不覆盖商务表</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>覆盖</t>
+          <t>状态</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>生文有线上刊例 56 款；其中已映射商务阶梯约 41 款，其余阶梯列标「—」询价</t>
+          <t>讨论定稿阶梯 · 待产品/商务确认后正式外发</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>覆盖</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>生文有线上刊例 56 款；其中已套公开分族/特例阶梯（非全原价）约 42 款</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>重建</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>python3 pricing/scripts/build_outward_quote_standard.py</t>
         </is>
@@ -761,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -769,7 +781,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
@@ -779,6 +791,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -788,10 +801,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>单位：USD / 百万 tokens　|　有效期：2026-08-31 24:00，过期作废，请联系商务获取最新报价。　阶梯达档：企业户单月累计消耗（按目录价计）；更大用量或合同价请联系商务。</t>
+          <t>单位：USD / 百万 tokens　|　有效期：2026-08-31 24:00，过期作废，请联系商务获取最新报价。　阶梯达档：企业户单月累计消耗（按目录价计）；更大用量或合同价请联系商务。　目录价含缓存列（无缓存刊例标「—」）。</t>
         </is>
       </c>
     </row>
@@ -823,34 +836,39 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
+          <t>目录价·缓存</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
           <t>≥$1k Plus</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>≥$5k Mid</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>≥$10k Growth</t>
         </is>
       </c>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="6" t="n"/>
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>≥$50k Scale</t>
         </is>
       </c>
-      <c r="M4" s="6" t="n"/>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>≥$100k Enterprise</t>
         </is>
       </c>
-      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="7" t="n"/>
@@ -858,52 +876,53 @@
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>输出</t>
         </is>
@@ -937,50 +956,55 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>1.8 (9折)</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>7.2 (9折)</t>
+          <t>1.76 (8.8折)</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
+          <t>7.04 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
           <t>1.7 (8.5折)</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>6.8 (8.5折)</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>1.64 (8.2折)</t>
         </is>
       </c>
-      <c r="K6" s="11" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>6.56 (8.2折)</t>
         </is>
       </c>
-      <c r="L6" s="11" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>1.52 (7.6折)</t>
         </is>
       </c>
-      <c r="M6" s="11" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>6.08 (7.6折)</t>
         </is>
       </c>
-      <c r="N6" s="11" t="inlineStr">
+      <c r="O6" s="11" t="inlineStr">
         <is>
           <t>1.44 (7.2折)</t>
         </is>
       </c>
-      <c r="O6" s="11" t="inlineStr">
+      <c r="P6" s="11" t="inlineStr">
         <is>
           <t>5.76 (7.2折)</t>
         </is>
@@ -1010,50 +1034,55 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>2.25 (9折)</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
-          <t>9 (9折)</t>
+          <t>2.2 (8.8折)</t>
         </is>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
+          <t>8.8 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
           <t>2.125 (8.5折)</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr">
+      <c r="J7" s="14" t="inlineStr">
         <is>
           <t>8.5 (8.5折)</t>
         </is>
       </c>
-      <c r="J7" s="14" t="inlineStr">
+      <c r="K7" s="14" t="inlineStr">
         <is>
           <t>2.05 (8.2折)</t>
         </is>
       </c>
-      <c r="K7" s="14" t="inlineStr">
+      <c r="L7" s="14" t="inlineStr">
         <is>
           <t>8.2 (8.2折)</t>
         </is>
       </c>
-      <c r="L7" s="14" t="inlineStr">
+      <c r="M7" s="14" t="inlineStr">
         <is>
           <t>1.9 (7.6折)</t>
         </is>
       </c>
-      <c r="M7" s="14" t="inlineStr">
+      <c r="N7" s="14" t="inlineStr">
         <is>
           <t>7.6 (7.6折)</t>
         </is>
       </c>
-      <c r="N7" s="14" t="inlineStr">
+      <c r="O7" s="14" t="inlineStr">
         <is>
           <t>1.8 (7.2折)</t>
         </is>
       </c>
-      <c r="O7" s="14" t="inlineStr">
+      <c r="P7" s="14" t="inlineStr">
         <is>
           <t>7.2 (7.2折)</t>
         </is>
@@ -1083,50 +1112,55 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>1.125 (9折)</t>
+          <t>0.125</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>9 (9折)</t>
+          <t>1.1 (8.8折)</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
+          <t>8.8 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
           <t>1.0625 (8.5折)</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>8.5 (8.5折)</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>1.025 (8.2折)</t>
         </is>
       </c>
-      <c r="K8" s="11" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>8.2 (8.2折)</t>
         </is>
       </c>
-      <c r="L8" s="11" t="inlineStr">
+      <c r="M8" s="11" t="inlineStr">
         <is>
           <t>0.95 (7.6折)</t>
         </is>
       </c>
-      <c r="M8" s="11" t="inlineStr">
+      <c r="N8" s="11" t="inlineStr">
         <is>
           <t>7.6 (7.6折)</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
+      <c r="O8" s="11" t="inlineStr">
         <is>
           <t>0.9 (7.2折)</t>
         </is>
       </c>
-      <c r="O8" s="11" t="inlineStr">
+      <c r="P8" s="11" t="inlineStr">
         <is>
           <t>7.2 (7.2折)</t>
         </is>
@@ -1156,52 +1190,57 @@
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.005</t>
         </is>
       </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.044 (8.8折)</t>
         </is>
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.352 (8.8折)</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.0425 (8.5折)</t>
         </is>
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.34 (8.5折)</t>
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.041 (8.2折)</t>
         </is>
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.328 (8.2折)</t>
         </is>
       </c>
       <c r="M9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.038 (7.6折)</t>
         </is>
       </c>
       <c r="N9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.304 (7.6折)</t>
         </is>
       </c>
       <c r="O9" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.036 (7.2折)</t>
+        </is>
+      </c>
+      <c r="P9" s="14" t="inlineStr">
+        <is>
+          <t>0.288 (7.2折)</t>
         </is>
       </c>
     </row>
@@ -1229,50 +1268,55 @@
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>1.125 (9折)</t>
+          <t>0.125</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>9 (9折)</t>
+          <t>1.1 (8.8折)</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
+          <t>8.8 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
           <t>1.0625 (8.5折)</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>8.5 (8.5折)</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>1.025 (8.2折)</t>
         </is>
       </c>
-      <c r="K10" s="11" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>8.2 (8.2折)</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr">
+      <c r="M10" s="11" t="inlineStr">
         <is>
           <t>0.95 (7.6折)</t>
         </is>
       </c>
-      <c r="M10" s="11" t="inlineStr">
+      <c r="N10" s="11" t="inlineStr">
         <is>
           <t>7.6 (7.6折)</t>
         </is>
       </c>
-      <c r="N10" s="11" t="inlineStr">
+      <c r="O10" s="11" t="inlineStr">
         <is>
           <t>0.9 (7.2折)</t>
         </is>
       </c>
-      <c r="O10" s="11" t="inlineStr">
+      <c r="P10" s="11" t="inlineStr">
         <is>
           <t>7.2 (7.2折)</t>
         </is>
@@ -1302,50 +1346,55 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>1.575 (9折)</t>
+          <t>0.175</t>
         </is>
       </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
-          <t>12.6 (9折)</t>
+          <t>1.54 (8.8折)</t>
         </is>
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
+          <t>12.32 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
           <t>1.4875 (8.5折)</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr">
+      <c r="J11" s="14" t="inlineStr">
         <is>
           <t>11.9 (8.5折)</t>
         </is>
       </c>
-      <c r="J11" s="14" t="inlineStr">
+      <c r="K11" s="14" t="inlineStr">
         <is>
           <t>1.435 (8.2折)</t>
         </is>
       </c>
-      <c r="K11" s="14" t="inlineStr">
+      <c r="L11" s="14" t="inlineStr">
         <is>
           <t>11.48 (8.2折)</t>
         </is>
       </c>
-      <c r="L11" s="14" t="inlineStr">
+      <c r="M11" s="14" t="inlineStr">
         <is>
           <t>1.33 (7.6折)</t>
         </is>
       </c>
-      <c r="M11" s="14" t="inlineStr">
+      <c r="N11" s="14" t="inlineStr">
         <is>
           <t>10.64 (7.6折)</t>
         </is>
       </c>
-      <c r="N11" s="14" t="inlineStr">
+      <c r="O11" s="14" t="inlineStr">
         <is>
           <t>1.26 (7.2折)</t>
         </is>
       </c>
-      <c r="O11" s="14" t="inlineStr">
+      <c r="P11" s="14" t="inlineStr">
         <is>
           <t>10.08 (7.2折)</t>
         </is>
@@ -1375,50 +1424,55 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>1.575 (9折)</t>
+          <t>0.175</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>12.6 (9折)</t>
+          <t>1.54 (8.8折)</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
+          <t>12.32 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
           <t>1.4875 (8.5折)</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>11.9 (8.5折)</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>1.435 (8.2折)</t>
         </is>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>11.48 (8.2折)</t>
         </is>
       </c>
-      <c r="L12" s="11" t="inlineStr">
+      <c r="M12" s="11" t="inlineStr">
         <is>
           <t>1.33 (7.6折)</t>
         </is>
       </c>
-      <c r="M12" s="11" t="inlineStr">
+      <c r="N12" s="11" t="inlineStr">
         <is>
           <t>10.64 (7.6折)</t>
         </is>
       </c>
-      <c r="N12" s="11" t="inlineStr">
+      <c r="O12" s="11" t="inlineStr">
         <is>
           <t>1.26 (7.2折)</t>
         </is>
       </c>
-      <c r="O12" s="11" t="inlineStr">
+      <c r="P12" s="11" t="inlineStr">
         <is>
           <t>10.08 (7.2折)</t>
         </is>
@@ -1448,50 +1502,55 @@
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>2.25 (9折)</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
-          <t>13.5 (9折)</t>
+          <t>2.2 (8.8折)</t>
         </is>
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
+          <t>13.2 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
           <t>2.125 (8.5折)</t>
         </is>
       </c>
-      <c r="I13" s="14" t="inlineStr">
+      <c r="J13" s="14" t="inlineStr">
         <is>
           <t>12.75 (8.5折)</t>
         </is>
       </c>
-      <c r="J13" s="14" t="inlineStr">
+      <c r="K13" s="14" t="inlineStr">
         <is>
           <t>2.05 (8.2折)</t>
         </is>
       </c>
-      <c r="K13" s="14" t="inlineStr">
+      <c r="L13" s="14" t="inlineStr">
         <is>
           <t>12.3 (8.2折)</t>
         </is>
       </c>
-      <c r="L13" s="14" t="inlineStr">
+      <c r="M13" s="14" t="inlineStr">
         <is>
           <t>1.9 (7.6折)</t>
         </is>
       </c>
-      <c r="M13" s="14" t="inlineStr">
+      <c r="N13" s="14" t="inlineStr">
         <is>
           <t>11.4 (7.6折)</t>
         </is>
       </c>
-      <c r="N13" s="14" t="inlineStr">
+      <c r="O13" s="14" t="inlineStr">
         <is>
           <t>1.8 (7.2折)</t>
         </is>
       </c>
-      <c r="O13" s="14" t="inlineStr">
+      <c r="P13" s="14" t="inlineStr">
         <is>
           <t>10.8 (7.2折)</t>
         </is>
@@ -1521,50 +1580,55 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>0.675 (9折)</t>
+          <t>0.075</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>4.05 (9折)</t>
+          <t>0.66 (8.8折)</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
+          <t>3.96 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
           <t>0.6375 (8.5折)</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr">
         <is>
           <t>3.825 (8.5折)</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>0.615 (8.2折)</t>
         </is>
       </c>
-      <c r="K14" s="11" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>3.69 (8.2折)</t>
         </is>
       </c>
-      <c r="L14" s="11" t="inlineStr">
+      <c r="M14" s="11" t="inlineStr">
         <is>
           <t>0.57 (7.6折)</t>
         </is>
       </c>
-      <c r="M14" s="11" t="inlineStr">
+      <c r="N14" s="11" t="inlineStr">
         <is>
           <t>3.42 (7.6折)</t>
         </is>
       </c>
-      <c r="N14" s="11" t="inlineStr">
+      <c r="O14" s="11" t="inlineStr">
         <is>
           <t>0.54 (7.2折)</t>
         </is>
       </c>
-      <c r="O14" s="11" t="inlineStr">
+      <c r="P14" s="11" t="inlineStr">
         <is>
           <t>3.24 (7.2折)</t>
         </is>
@@ -1594,50 +1658,55 @@
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>0.18 (9折)</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
-          <t>1.125 (9折)</t>
+          <t>0.176 (8.8折)</t>
         </is>
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
+          <t>1.1 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
+        <is>
           <t>0.17 (8.5折)</t>
         </is>
       </c>
-      <c r="I15" s="14" t="inlineStr">
+      <c r="J15" s="14" t="inlineStr">
         <is>
           <t>1.0625 (8.5折)</t>
         </is>
       </c>
-      <c r="J15" s="14" t="inlineStr">
+      <c r="K15" s="14" t="inlineStr">
         <is>
           <t>0.164 (8.2折)</t>
         </is>
       </c>
-      <c r="K15" s="14" t="inlineStr">
+      <c r="L15" s="14" t="inlineStr">
         <is>
           <t>1.025 (8.2折)</t>
         </is>
       </c>
-      <c r="L15" s="14" t="inlineStr">
+      <c r="M15" s="14" t="inlineStr">
         <is>
           <t>0.152 (7.6折)</t>
         </is>
       </c>
-      <c r="M15" s="14" t="inlineStr">
+      <c r="N15" s="14" t="inlineStr">
         <is>
           <t>0.95 (7.6折)</t>
         </is>
       </c>
-      <c r="N15" s="14" t="inlineStr">
+      <c r="O15" s="14" t="inlineStr">
         <is>
           <t>0.144 (7.2折)</t>
         </is>
       </c>
-      <c r="O15" s="14" t="inlineStr">
+      <c r="P15" s="14" t="inlineStr">
         <is>
           <t>0.9 (7.2折)</t>
         </is>
@@ -1667,52 +1736,57 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>30 (原价)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>180 (原价)</t>
+          <t>28.8 (9.6折)</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>30 (原价)</t>
+          <t>172.8 (9.6折)</t>
         </is>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>180 (原价)</t>
+          <t>28.2 (9.4折)</t>
         </is>
       </c>
       <c r="J16" s="11" t="inlineStr">
         <is>
-          <t>29.4 (9.8折)</t>
+          <t>169.2 (9.4折)</t>
         </is>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>176.4 (9.8折)</t>
+          <t>27.6 (9.2折)</t>
         </is>
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>27.3 (9.1折)</t>
+          <t>165.6 (9.2折)</t>
         </is>
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>163.8 (9.1折)</t>
+          <t>26.4 (8.8折)</t>
         </is>
       </c>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>26.1 (8.7折)</t>
+          <t>158.4 (8.8折)</t>
         </is>
       </c>
       <c r="O16" s="11" t="inlineStr">
         <is>
-          <t>156.6 (8.7折)</t>
+          <t>25.5 (8.5折)</t>
+        </is>
+      </c>
+      <c r="P16" s="11" t="inlineStr">
+        <is>
+          <t>153 (8.5折)</t>
         </is>
       </c>
     </row>
@@ -1740,52 +1814,57 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>30 (原价)</t>
+          <t>4.8 (9.6折)</t>
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>28.8 (9.6折)</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t>30 (原价)</t>
+          <t>4.7 (9.4折)</t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>4.9 (9.8折)</t>
+          <t>28.2 (9.4折)</t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>29.4 (9.8折)</t>
+          <t>4.6 (9.2折)</t>
         </is>
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>4.55 (9.1折)</t>
+          <t>27.6 (9.2折)</t>
         </is>
       </c>
       <c r="M17" s="14" t="inlineStr">
         <is>
-          <t>27.3 (9.1折)</t>
+          <t>4.4 (8.8折)</t>
         </is>
       </c>
       <c r="N17" s="14" t="inlineStr">
         <is>
-          <t>4.35 (8.7折)</t>
+          <t>26.4 (8.8折)</t>
         </is>
       </c>
       <c r="O17" s="14" t="inlineStr">
         <is>
-          <t>26.1 (8.7折)</t>
+          <t>4.25 (8.5折)</t>
+        </is>
+      </c>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>25.5 (8.5折)</t>
         </is>
       </c>
     </row>
@@ -1817,52 +1896,57 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.9 (9.8折)</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>24.5 (9.8折)</t>
         </is>
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.75 (9.5折)</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr">
         <is>
-          <t>4.9 (9.8折)</t>
+          <t>23.75 (9.5折)</t>
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>24.5 (9.8折)</t>
+          <t>4.6 (9.2折)</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>4.55 (9.1折)</t>
+          <t>23 (9.2折)</t>
         </is>
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>22.75 (9.1折)</t>
+          <t>4.5 (9折)</t>
         </is>
       </c>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>4.35 (8.7折)</t>
+          <t>22.5 (9折)</t>
         </is>
       </c>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>21.75 (8.7折)</t>
+          <t>4.4 (8.8折)</t>
+        </is>
+      </c>
+      <c r="P18" s="11" t="inlineStr">
+        <is>
+          <t>22 (8.8折)</t>
         </is>
       </c>
     </row>
@@ -1890,52 +1974,57 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.9 (9.8折)</t>
         </is>
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>24.5 (9.8折)</t>
         </is>
       </c>
       <c r="I19" s="14" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.75 (9.5折)</t>
         </is>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>4.9 (9.8折)</t>
+          <t>23.75 (9.5折)</t>
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>24.5 (9.8折)</t>
+          <t>4.6 (9.2折)</t>
         </is>
       </c>
       <c r="L19" s="14" t="inlineStr">
         <is>
-          <t>4.55 (9.1折)</t>
+          <t>23 (9.2折)</t>
         </is>
       </c>
       <c r="M19" s="14" t="inlineStr">
         <is>
-          <t>22.75 (9.1折)</t>
+          <t>4.5 (9折)</t>
         </is>
       </c>
       <c r="N19" s="14" t="inlineStr">
         <is>
-          <t>4.35 (8.7折)</t>
+          <t>22.5 (9折)</t>
         </is>
       </c>
       <c r="O19" s="14" t="inlineStr">
         <is>
-          <t>21.75 (8.7折)</t>
+          <t>4.4 (8.8折)</t>
+        </is>
+      </c>
+      <c r="P19" s="14" t="inlineStr">
+        <is>
+          <t>22 (8.8折)</t>
         </is>
       </c>
     </row>
@@ -1963,52 +2052,57 @@
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.9 (9.8折)</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>5 (原价)</t>
+          <t>24.5 (9.8折)</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>25 (原价)</t>
+          <t>4.75 (9.5折)</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr">
         <is>
-          <t>4.9 (9.8折)</t>
+          <t>23.75 (9.5折)</t>
         </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>24.5 (9.8折)</t>
+          <t>4.6 (9.2折)</t>
         </is>
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>4.55 (9.1折)</t>
+          <t>23 (9.2折)</t>
         </is>
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>22.75 (9.1折)</t>
+          <t>4.5 (9折)</t>
         </is>
       </c>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>4.35 (8.7折)</t>
+          <t>22.5 (9折)</t>
         </is>
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
-          <t>21.75 (8.7折)</t>
+          <t>4.4 (8.8折)</t>
+        </is>
+      </c>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>22 (8.8折)</t>
         </is>
       </c>
     </row>
@@ -2036,52 +2130,57 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>3 (原价)</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>15 (原价)</t>
+          <t>2.94 (9.8折)</t>
         </is>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>3 (原价)</t>
+          <t>14.7 (9.8折)</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>15 (原价)</t>
+          <t>2.85 (9.5折)</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>2.94 (9.8折)</t>
+          <t>14.25 (9.5折)</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>14.7 (9.8折)</t>
+          <t>2.76 (9.2折)</t>
         </is>
       </c>
       <c r="L21" s="14" t="inlineStr">
         <is>
-          <t>2.73 (9.1折)</t>
+          <t>13.8 (9.2折)</t>
         </is>
       </c>
       <c r="M21" s="14" t="inlineStr">
         <is>
-          <t>13.65 (9.1折)</t>
+          <t>2.7 (9折)</t>
         </is>
       </c>
       <c r="N21" s="14" t="inlineStr">
         <is>
-          <t>2.61 (8.7折)</t>
+          <t>13.5 (9折)</t>
         </is>
       </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
-          <t>13.05 (8.7折)</t>
+          <t>2.64 (8.8折)</t>
+        </is>
+      </c>
+      <c r="P21" s="14" t="inlineStr">
+        <is>
+          <t>13.2 (8.8折)</t>
         </is>
       </c>
     </row>
@@ -2113,50 +2212,55 @@
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>0.291 (9.7折)</t>
+          <t>0.03</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>2.425 (9.7折)</t>
+          <t>0.27 (9折)</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>0.276 (9.2折)</t>
+          <t>2.25 (9折)</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>2.3 (9.2折)</t>
+          <t>0.264 (8.8折)</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr">
         <is>
-          <t>0.264 (8.8折)</t>
+          <t>2.2 (8.8折)</t>
         </is>
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>2.2 (8.8折)</t>
+          <t>0.255 (8.5折)</t>
         </is>
       </c>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>0.246 (8.2折)</t>
+          <t>2.125 (8.5折)</t>
         </is>
       </c>
       <c r="M22" s="11" t="inlineStr">
         <is>
-          <t>2.05 (8.2折)</t>
+          <t>0.24 (8折)</t>
         </is>
       </c>
       <c r="N22" s="11" t="inlineStr">
         <is>
+          <t>2 (8折)</t>
+        </is>
+      </c>
+      <c r="O22" s="11" t="inlineStr">
+        <is>
           <t>0.234 (7.8折)</t>
         </is>
       </c>
-      <c r="O22" s="11" t="inlineStr">
+      <c r="P22" s="11" t="inlineStr">
         <is>
           <t>1.95 (7.8折)</t>
         </is>
@@ -2186,50 +2290,55 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>0.097 (9.7折)</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>0.388 (9.7折)</t>
+          <t>0.09 (9折)</t>
         </is>
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>0.092 (9.2折)</t>
+          <t>0.36 (9折)</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>0.368 (9.2折)</t>
+          <t>0.088 (8.8折)</t>
         </is>
       </c>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>0.088 (8.8折)</t>
+          <t>0.352 (8.8折)</t>
         </is>
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>0.352 (8.8折)</t>
+          <t>0.085 (8.5折)</t>
         </is>
       </c>
       <c r="L23" s="14" t="inlineStr">
         <is>
-          <t>0.082 (8.2折)</t>
+          <t>0.34 (8.5折)</t>
         </is>
       </c>
       <c r="M23" s="14" t="inlineStr">
         <is>
-          <t>0.328 (8.2折)</t>
+          <t>0.08 (8折)</t>
         </is>
       </c>
       <c r="N23" s="14" t="inlineStr">
         <is>
+          <t>0.32 (8折)</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
           <t>0.078 (7.8折)</t>
         </is>
       </c>
-      <c r="O23" s="14" t="inlineStr">
+      <c r="P23" s="14" t="inlineStr">
         <is>
           <t>0.312 (7.8折)</t>
         </is>
@@ -2259,52 +2368,57 @@
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>0.1 (原价)</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>0.4 (原价)</t>
+          <t>0.092 (9.2折)</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>0.098 (9.8折)</t>
+          <t>0.368 (9.2折)</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>0.392 (9.8折)</t>
+          <t>0.09 (9折)</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr">
         <is>
-          <t>0.094 (9.4折)</t>
+          <t>0.36 (9折)</t>
         </is>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>0.376 (9.4折)</t>
+          <t>0.087 (8.7折)</t>
         </is>
       </c>
       <c r="L24" s="11" t="inlineStr">
         <is>
-          <t>0.088 (8.8折)</t>
+          <t>0.348 (8.7折)</t>
         </is>
       </c>
       <c r="M24" s="11" t="inlineStr">
         <is>
-          <t>0.352 (8.8折)</t>
+          <t>0.085 (8.5折)</t>
         </is>
       </c>
       <c r="N24" s="11" t="inlineStr">
         <is>
-          <t>0.083 (8.3折)</t>
+          <t>0.34 (8.5折)</t>
         </is>
       </c>
       <c r="O24" s="11" t="inlineStr">
         <is>
-          <t>0.332 (8.3折)</t>
+          <t>0.082 (8.2折)</t>
+        </is>
+      </c>
+      <c r="P24" s="11" t="inlineStr">
+        <is>
+          <t>0.328 (8.2折)</t>
         </is>
       </c>
     </row>
@@ -2332,50 +2446,55 @@
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>1.2125 (9.7折)</t>
+          <t>0.125</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>9.7 (9.7折)</t>
+          <t>1.125 (9折)</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>1.15 (9.2折)</t>
+          <t>9 (9折)</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>9.2 (9.2折)</t>
+          <t>1.1 (8.8折)</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>1.1 (8.8折)</t>
+          <t>8.8 (8.8折)</t>
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>8.8 (8.8折)</t>
+          <t>1.0625 (8.5折)</t>
         </is>
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>1.025 (8.2折)</t>
+          <t>8.5 (8.5折)</t>
         </is>
       </c>
       <c r="M25" s="14" t="inlineStr">
         <is>
-          <t>8.2 (8.2折)</t>
+          <t>1 (8折)</t>
         </is>
       </c>
       <c r="N25" s="14" t="inlineStr">
         <is>
+          <t>8 (8折)</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
           <t>0.975 (7.8折)</t>
         </is>
       </c>
-      <c r="O25" s="14" t="inlineStr">
+      <c r="P25" s="14" t="inlineStr">
         <is>
           <t>7.8 (7.8折)</t>
         </is>
@@ -2405,50 +2524,55 @@
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>0.485 (9.7折)</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>2.91 (9.7折)</t>
+          <t>0.45 (9折)</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>0.46 (9.2折)</t>
+          <t>2.7 (9折)</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>2.76 (9.2折)</t>
+          <t>0.44 (8.8折)</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr">
         <is>
-          <t>0.44 (8.8折)</t>
+          <t>2.64 (8.8折)</t>
         </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>2.64 (8.8折)</t>
+          <t>0.425 (8.5折)</t>
         </is>
       </c>
       <c r="L26" s="11" t="inlineStr">
         <is>
-          <t>0.41 (8.2折)</t>
+          <t>2.55 (8.5折)</t>
         </is>
       </c>
       <c r="M26" s="11" t="inlineStr">
         <is>
-          <t>2.46 (8.2折)</t>
+          <t>0.4 (8折)</t>
         </is>
       </c>
       <c r="N26" s="11" t="inlineStr">
         <is>
+          <t>2.4 (8折)</t>
+        </is>
+      </c>
+      <c r="O26" s="11" t="inlineStr">
+        <is>
           <t>0.39 (7.8折)</t>
         </is>
       </c>
-      <c r="O26" s="11" t="inlineStr">
+      <c r="P26" s="11" t="inlineStr">
         <is>
           <t>2.34 (7.8折)</t>
         </is>
@@ -2478,50 +2602,55 @@
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>0.2425 (9.7折)</t>
+          <t>0.025</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>1.455 (9.7折)</t>
+          <t>0.225 (9折)</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>0.23 (9.2折)</t>
+          <t>1.35 (9折)</t>
         </is>
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>1.38 (9.2折)</t>
+          <t>0.22 (8.8折)</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>0.22 (8.8折)</t>
+          <t>1.32 (8.8折)</t>
         </is>
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>1.32 (8.8折)</t>
+          <t>0.2125 (8.5折)</t>
         </is>
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
-          <t>0.205 (8.2折)</t>
+          <t>1.275 (8.5折)</t>
         </is>
       </c>
       <c r="M27" s="14" t="inlineStr">
         <is>
-          <t>1.23 (8.2折)</t>
+          <t>0.2 (8折)</t>
         </is>
       </c>
       <c r="N27" s="14" t="inlineStr">
         <is>
+          <t>1.2 (8折)</t>
+        </is>
+      </c>
+      <c r="O27" s="14" t="inlineStr">
+        <is>
           <t>0.195 (7.8折)</t>
         </is>
       </c>
-      <c r="O27" s="14" t="inlineStr">
+      <c r="P27" s="14" t="inlineStr">
         <is>
           <t>1.17 (7.8折)</t>
         </is>
@@ -2551,50 +2680,55 @@
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>1.94 (9.7折)</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>11.64 (9.7折)</t>
+          <t>1.8 (9折)</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>1.84 (9.2折)</t>
+          <t>10.8 (9折)</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>11.04 (9.2折)</t>
+          <t>1.76 (8.8折)</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>1.76 (8.8折)</t>
+          <t>10.56 (8.8折)</t>
         </is>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>10.56 (8.8折)</t>
+          <t>1.7 (8.5折)</t>
         </is>
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>1.64 (8.2折)</t>
+          <t>10.2 (8.5折)</t>
         </is>
       </c>
       <c r="M28" s="11" t="inlineStr">
         <is>
-          <t>9.84 (8.2折)</t>
+          <t>1.6 (8折)</t>
         </is>
       </c>
       <c r="N28" s="11" t="inlineStr">
         <is>
+          <t>9.6 (8折)</t>
+        </is>
+      </c>
+      <c r="O28" s="11" t="inlineStr">
+        <is>
           <t>1.56 (7.8折)</t>
         </is>
       </c>
-      <c r="O28" s="11" t="inlineStr">
+      <c r="P28" s="11" t="inlineStr">
         <is>
           <t>9.36 (7.8折)</t>
         </is>
@@ -2624,50 +2758,55 @@
       </c>
       <c r="F29" s="14" t="inlineStr">
         <is>
-          <t>1.455 (9.7折)</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>8.73 (9.7折)</t>
+          <t>1.35 (9折)</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>1.38 (9.2折)</t>
+          <t>8.1 (9折)</t>
         </is>
       </c>
       <c r="I29" s="14" t="inlineStr">
         <is>
-          <t>8.28 (9.2折)</t>
+          <t>1.32 (8.8折)</t>
         </is>
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>1.32 (8.8折)</t>
+          <t>7.92 (8.8折)</t>
         </is>
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>7.92 (8.8折)</t>
+          <t>1.275 (8.5折)</t>
         </is>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>1.23 (8.2折)</t>
+          <t>7.65 (8.5折)</t>
         </is>
       </c>
       <c r="M29" s="14" t="inlineStr">
         <is>
-          <t>7.38 (8.2折)</t>
+          <t>1.2 (8折)</t>
         </is>
       </c>
       <c r="N29" s="14" t="inlineStr">
         <is>
+          <t>7.2 (8折)</t>
+        </is>
+      </c>
+      <c r="O29" s="14" t="inlineStr">
+        <is>
           <t>1.17 (7.8折)</t>
         </is>
       </c>
-      <c r="O29" s="14" t="inlineStr">
+      <c r="P29" s="14" t="inlineStr">
         <is>
           <t>7.02 (7.8折)</t>
         </is>
@@ -2701,50 +2840,55 @@
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>0.298461 (9.7折)</t>
+          <t>0.061538</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>0.447692 (9.7折)</t>
+          <t>0.276923 (9折)</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>0.283077 (9.2折)</t>
+          <t>0.415384 (9折)</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>0.424615 (9.2折)</t>
+          <t>0.270769 (8.8折)</t>
         </is>
       </c>
       <c r="J30" s="11" t="inlineStr">
         <is>
-          <t>0.270769 (8.8折)</t>
+          <t>0.406153 (8.8折)</t>
         </is>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>0.406153 (8.8折)</t>
+          <t>0.261538 (8.5折)</t>
         </is>
       </c>
       <c r="L30" s="11" t="inlineStr">
         <is>
-          <t>0.252307 (8.2折)</t>
+          <t>0.392307 (8.5折)</t>
         </is>
       </c>
       <c r="M30" s="11" t="inlineStr">
         <is>
-          <t>0.378461 (8.2折)</t>
+          <t>0.246154 (8折)</t>
         </is>
       </c>
       <c r="N30" s="11" t="inlineStr">
         <is>
+          <t>0.36923 (8折)</t>
+        </is>
+      </c>
+      <c r="O30" s="11" t="inlineStr">
+        <is>
           <t>0.24 (7.8折)</t>
         </is>
       </c>
-      <c r="O30" s="11" t="inlineStr">
+      <c r="P30" s="11" t="inlineStr">
         <is>
           <t>0.36 (7.8折)</t>
         </is>
@@ -2774,50 +2918,55 @@
       </c>
       <c r="F31" s="14" t="inlineStr">
         <is>
-          <t>0.149231 (9.7折)</t>
+          <t>0.003077</t>
         </is>
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>0.298461 (9.7折)</t>
+          <t>0.138461 (9折)</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>0.141538 (9.2折)</t>
+          <t>0.276923 (9折)</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>0.283077 (9.2折)</t>
+          <t>0.135384 (8.8折)</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
-          <t>0.135384 (8.8折)</t>
+          <t>0.270769 (8.8折)</t>
         </is>
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>0.270769 (8.8折)</t>
+          <t>0.130769 (8.5折)</t>
         </is>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>0.126154 (8.2折)</t>
+          <t>0.261538 (8.5折)</t>
         </is>
       </c>
       <c r="M31" s="14" t="inlineStr">
         <is>
-          <t>0.252307 (8.2折)</t>
+          <t>0.123077 (8折)</t>
         </is>
       </c>
       <c r="N31" s="14" t="inlineStr">
         <is>
+          <t>0.246154 (8折)</t>
+        </is>
+      </c>
+      <c r="O31" s="14" t="inlineStr">
+        <is>
           <t>0.12 (7.8折)</t>
         </is>
       </c>
-      <c r="O31" s="14" t="inlineStr">
+      <c r="P31" s="14" t="inlineStr">
         <is>
           <t>0.24 (7.8折)</t>
         </is>
@@ -2847,52 +2996,57 @@
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.003846</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.461538 (原价)</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.923077 (原价)</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.461538 (原价)</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.923077 (原价)</t>
         </is>
       </c>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.461538 (原价)</t>
         </is>
       </c>
       <c r="L32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.923077 (原价)</t>
         </is>
       </c>
       <c r="M32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.461538 (原价)</t>
         </is>
       </c>
       <c r="N32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.923077 (原价)</t>
         </is>
       </c>
       <c r="O32" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.461538 (原价)</t>
+        </is>
+      </c>
+      <c r="P32" s="11" t="inlineStr">
+        <is>
+          <t>0.923077 (原价)</t>
         </is>
       </c>
     </row>
@@ -2924,50 +3078,55 @@
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>0.596923 (9.7折)</t>
+          <t>0.107692</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>3.133846 (9.7折)</t>
+          <t>0.553847 (9折)</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>0.566154 (9.2折)</t>
+          <t>2.907692 (9折)</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>2.972307 (9.2折)</t>
+          <t>0.541539 (8.8折)</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>0.541539 (8.8折)</t>
+          <t>2.843077 (8.8折)</t>
         </is>
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>2.843077 (8.8折)</t>
+          <t>0.523077 (8.5折)</t>
         </is>
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>0.504616 (8.2折)</t>
+          <t>2.746154 (8.5折)</t>
         </is>
       </c>
       <c r="M33" s="14" t="inlineStr">
         <is>
-          <t>2.649231 (8.2折)</t>
+          <t>0.492308 (8折)</t>
         </is>
       </c>
       <c r="N33" s="14" t="inlineStr">
         <is>
+          <t>2.584615 (8折)</t>
+        </is>
+      </c>
+      <c r="O33" s="14" t="inlineStr">
+        <is>
           <t>0.48 (7.8折)</t>
         </is>
       </c>
-      <c r="O33" s="14" t="inlineStr">
+      <c r="P33" s="14" t="inlineStr">
         <is>
           <t>2.52 (7.8折)</t>
         </is>
@@ -2997,50 +3156,55 @@
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
-          <t>0.97 (9.7折)</t>
+          <t>0.169231</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>4.029231 (9.7折)</t>
+          <t>0.9 (9折)</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>0.92 (9.2折)</t>
+          <t>3.738461 (9折)</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>3.821538 (9.2折)</t>
+          <t>0.88 (8.8折)</t>
         </is>
       </c>
       <c r="J34" s="11" t="inlineStr">
         <is>
-          <t>0.88 (8.8折)</t>
+          <t>3.655384 (8.8折)</t>
         </is>
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>3.655384 (8.8折)</t>
+          <t>0.85 (8.5折)</t>
         </is>
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
-          <t>0.82 (8.2折)</t>
+          <t>3.530769 (8.5折)</t>
         </is>
       </c>
       <c r="M34" s="11" t="inlineStr">
         <is>
-          <t>3.406154 (8.2折)</t>
+          <t>0.8 (8折)</t>
         </is>
       </c>
       <c r="N34" s="11" t="inlineStr">
         <is>
+          <t>3.323077 (8折)</t>
+        </is>
+      </c>
+      <c r="O34" s="11" t="inlineStr">
+        <is>
           <t>0.78 (7.8折)</t>
         </is>
       </c>
-      <c r="O34" s="11" t="inlineStr">
+      <c r="P34" s="11" t="inlineStr">
         <is>
           <t>3.24 (7.8折)</t>
         </is>
@@ -3070,50 +3234,55 @@
       </c>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>0.97 (9.7折)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>4.029231 (9.7折)</t>
+          <t>0.9 (9折)</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>0.92 (9.2折)</t>
+          <t>3.738461 (9折)</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>3.821538 (9.2折)</t>
+          <t>0.88 (8.8折)</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>0.88 (8.8折)</t>
+          <t>3.655384 (8.8折)</t>
         </is>
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>3.655384 (8.8折)</t>
+          <t>0.85 (8.5折)</t>
         </is>
       </c>
       <c r="L35" s="14" t="inlineStr">
         <is>
-          <t>0.82 (8.2折)</t>
+          <t>3.530769 (8.5折)</t>
         </is>
       </c>
       <c r="M35" s="14" t="inlineStr">
         <is>
-          <t>3.406154 (8.2折)</t>
+          <t>0.8 (8折)</t>
         </is>
       </c>
       <c r="N35" s="14" t="inlineStr">
         <is>
+          <t>3.323077 (8折)</t>
+        </is>
+      </c>
+      <c r="O35" s="14" t="inlineStr">
+        <is>
           <t>0.78 (7.8折)</t>
         </is>
       </c>
-      <c r="O35" s="14" t="inlineStr">
+      <c r="P35" s="14" t="inlineStr">
         <is>
           <t>3.24 (7.8折)</t>
         </is>
@@ -3143,52 +3312,57 @@
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 (原价)</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.307692 (原价)</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 (原价)</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.307692 (原价)</t>
         </is>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 (原价)</t>
         </is>
       </c>
       <c r="L36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.307692 (原价)</t>
         </is>
       </c>
       <c r="M36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 (原价)</t>
         </is>
       </c>
       <c r="N36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8.307692 (原价)</t>
         </is>
       </c>
       <c r="O36" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2 (原价)</t>
+        </is>
+      </c>
+      <c r="P36" s="11" t="inlineStr">
+        <is>
+          <t>8.307692 (原价)</t>
         </is>
       </c>
     </row>
@@ -3220,52 +3394,57 @@
       </c>
       <c r="F37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.032308</t>
         </is>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="L37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="M37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="N37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="O37" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
+        </is>
+      </c>
+      <c r="P37" s="14" t="inlineStr">
+        <is>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
     </row>
@@ -3293,52 +3472,57 @@
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.064615</t>
         </is>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="L38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="M38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="N38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="O38" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
+        </is>
+      </c>
+      <c r="P38" s="11" t="inlineStr">
+        <is>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
     </row>
@@ -3366,52 +3550,57 @@
       </c>
       <c r="F39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.064615</t>
         </is>
       </c>
       <c r="G39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="I39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="K39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="M39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
         </is>
       </c>
       <c r="N39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
       <c r="O39" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.323077 (原价)</t>
+        </is>
+      </c>
+      <c r="P39" s="14" t="inlineStr">
+        <is>
+          <t>1.292308 (原价)</t>
         </is>
       </c>
     </row>
@@ -3443,50 +3632,55 @@
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>0.596923 (9.7折)</t>
+          <t>0.153846</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>2.686154 (9.7折)</t>
+          <t>0.553847 (9折)</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>0.566154 (9.2折)</t>
+          <t>2.492308 (9折)</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>2.547693 (9.2折)</t>
+          <t>0.541539 (8.8折)</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
         <is>
-          <t>0.541539 (8.8折)</t>
+          <t>2.436923 (8.8折)</t>
         </is>
       </c>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>2.436923 (8.8折)</t>
+          <t>0.523077 (8.5折)</t>
         </is>
       </c>
       <c r="L40" s="11" t="inlineStr">
         <is>
-          <t>0.504616 (8.2折)</t>
+          <t>2.353846 (8.5折)</t>
         </is>
       </c>
       <c r="M40" s="11" t="inlineStr">
         <is>
-          <t>2.270769 (8.2折)</t>
+          <t>0.492308 (8折)</t>
         </is>
       </c>
       <c r="N40" s="11" t="inlineStr">
         <is>
+          <t>2.215385 (8折)</t>
+        </is>
+      </c>
+      <c r="O40" s="11" t="inlineStr">
+        <is>
           <t>0.48 (7.8折)</t>
         </is>
       </c>
-      <c r="O40" s="11" t="inlineStr">
+      <c r="P40" s="11" t="inlineStr">
         <is>
           <t>2.16 (7.8折)</t>
         </is>
@@ -3516,52 +3710,57 @@
       </c>
       <c r="F41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615</t>
         </is>
       </c>
       <c r="G41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="L41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="M41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="N41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="O41" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
+        </is>
+      </c>
+      <c r="P41" s="14" t="inlineStr">
+        <is>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
     </row>
@@ -3589,50 +3788,55 @@
       </c>
       <c r="F42" s="11" t="inlineStr">
         <is>
-          <t>0.895385 (9.7折)</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>3.581539 (9.7折)</t>
+          <t>0.830769 (9折)</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>0.849231 (9.2折)</t>
+          <t>3.323077 (9折)</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>3.396923 (9.2折)</t>
+          <t>0.812308 (8.8折)</t>
         </is>
       </c>
       <c r="J42" s="11" t="inlineStr">
         <is>
-          <t>0.812308 (8.8折)</t>
+          <t>3.249231 (8.8折)</t>
         </is>
       </c>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>3.249231 (8.8折)</t>
+          <t>0.784615 (8.5折)</t>
         </is>
       </c>
       <c r="L42" s="11" t="inlineStr">
         <is>
-          <t>0.756923 (8.2折)</t>
+          <t>3.138462 (8.5折)</t>
         </is>
       </c>
       <c r="M42" s="11" t="inlineStr">
         <is>
-          <t>3.027693 (8.2折)</t>
+          <t>0.738462 (8折)</t>
         </is>
       </c>
       <c r="N42" s="11" t="inlineStr">
         <is>
+          <t>2.953846 (8折)</t>
+        </is>
+      </c>
+      <c r="O42" s="11" t="inlineStr">
+        <is>
           <t>0.72 (7.8折)</t>
         </is>
       </c>
-      <c r="O42" s="11" t="inlineStr">
+      <c r="P42" s="11" t="inlineStr">
         <is>
           <t>2.88 (7.8折)</t>
         </is>
@@ -3662,50 +3866,55 @@
       </c>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>1.193846 (9.7折)</t>
+          <t>0.307692</t>
         </is>
       </c>
       <c r="G43" s="14" t="inlineStr">
         <is>
-          <t>4.178461 (9.7折)</t>
+          <t>1.107692 (9折)</t>
         </is>
       </c>
       <c r="H43" s="14" t="inlineStr">
         <is>
-          <t>1.132307 (9.2折)</t>
+          <t>3.876923 (9折)</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
         <is>
-          <t>3.963077 (9.2折)</t>
+          <t>1.083077 (8.8折)</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>1.083077 (8.8折)</t>
+          <t>3.790769 (8.8折)</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr">
         <is>
-          <t>3.790769 (8.8折)</t>
+          <t>1.046154 (8.5折)</t>
         </is>
       </c>
       <c r="L43" s="14" t="inlineStr">
         <is>
-          <t>1.009231 (8.2折)</t>
+          <t>3.661538 (8.5折)</t>
         </is>
       </c>
       <c r="M43" s="14" t="inlineStr">
         <is>
-          <t>3.532307 (8.2折)</t>
+          <t>0.984615 (8折)</t>
         </is>
       </c>
       <c r="N43" s="14" t="inlineStr">
         <is>
+          <t>3.446154 (8折)</t>
+        </is>
+      </c>
+      <c r="O43" s="14" t="inlineStr">
+        <is>
           <t>0.96 (7.8折)</t>
         </is>
       </c>
-      <c r="O43" s="14" t="inlineStr">
+      <c r="P43" s="14" t="inlineStr">
         <is>
           <t>3.36 (7.8折)</t>
         </is>
@@ -3735,52 +3944,57 @@
       </c>
       <c r="F44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615</t>
         </is>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="J44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="L44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="M44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
         </is>
       </c>
       <c r="N44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
       <c r="O44" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.769231 (原价)</t>
+        </is>
+      </c>
+      <c r="P44" s="11" t="inlineStr">
+        <is>
+          <t>3.384615 (原价)</t>
         </is>
       </c>
     </row>
@@ -3812,50 +4026,55 @@
       </c>
       <c r="F45" s="14" t="inlineStr">
         <is>
-          <t>0.020769 (9折)</t>
+          <t>0.004615</t>
         </is>
       </c>
       <c r="G45" s="14" t="inlineStr">
         <is>
-          <t>0.207692 (9折)</t>
+          <t>0.020308 (8.8折)</t>
         </is>
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
+          <t>0.203077 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
+        <is>
           <t>0.019615 (8.5折)</t>
         </is>
       </c>
-      <c r="I45" s="14" t="inlineStr">
+      <c r="J45" s="14" t="inlineStr">
         <is>
           <t>0.196154 (8.5折)</t>
         </is>
       </c>
-      <c r="J45" s="14" t="inlineStr">
+      <c r="K45" s="14" t="inlineStr">
         <is>
           <t>0.018923 (8.2折)</t>
         </is>
       </c>
-      <c r="K45" s="14" t="inlineStr">
+      <c r="L45" s="14" t="inlineStr">
         <is>
           <t>0.189231 (8.2折)</t>
         </is>
       </c>
-      <c r="L45" s="14" t="inlineStr">
+      <c r="M45" s="14" t="inlineStr">
         <is>
           <t>0.017539 (7.6折)</t>
         </is>
       </c>
-      <c r="M45" s="14" t="inlineStr">
+      <c r="N45" s="14" t="inlineStr">
         <is>
           <t>0.175384 (7.6折)</t>
         </is>
       </c>
-      <c r="N45" s="14" t="inlineStr">
+      <c r="O45" s="14" t="inlineStr">
         <is>
           <t>0.016615 (7.2折)</t>
         </is>
       </c>
-      <c r="O45" s="14" t="inlineStr">
+      <c r="P45" s="14" t="inlineStr">
         <is>
           <t>0.166154 (7.2折)</t>
         </is>
@@ -3885,50 +4104,55 @@
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>0.332308 (9折)</t>
+          <t>0.082759</t>
         </is>
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>1.329231 (9折)</t>
+          <t>0.324923 (8.8折)</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
+          <t>1.299692 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
           <t>0.313846 (8.5折)</t>
         </is>
       </c>
-      <c r="I46" s="11" t="inlineStr">
+      <c r="J46" s="11" t="inlineStr">
         <is>
           <t>1.255385 (8.5折)</t>
         </is>
       </c>
-      <c r="J46" s="11" t="inlineStr">
+      <c r="K46" s="11" t="inlineStr">
         <is>
           <t>0.302769 (8.2折)</t>
         </is>
       </c>
-      <c r="K46" s="11" t="inlineStr">
+      <c r="L46" s="11" t="inlineStr">
         <is>
           <t>1.211077 (8.2折)</t>
         </is>
       </c>
-      <c r="L46" s="11" t="inlineStr">
+      <c r="M46" s="11" t="inlineStr">
         <is>
           <t>0.280616 (7.6折)</t>
         </is>
       </c>
-      <c r="M46" s="11" t="inlineStr">
+      <c r="N46" s="11" t="inlineStr">
         <is>
           <t>1.122461 (7.6折)</t>
         </is>
       </c>
-      <c r="N46" s="11" t="inlineStr">
+      <c r="O46" s="11" t="inlineStr">
         <is>
           <t>0.265846 (7.2折)</t>
         </is>
       </c>
-      <c r="O46" s="11" t="inlineStr">
+      <c r="P46" s="11" t="inlineStr">
         <is>
           <t>1.063385 (7.2折)</t>
         </is>
@@ -3958,50 +4182,55 @@
       </c>
       <c r="F47" s="14" t="inlineStr">
         <is>
-          <t>0.110769 (9折)</t>
+          <t>0.024615</t>
         </is>
       </c>
       <c r="G47" s="14" t="inlineStr">
         <is>
-          <t>0.276923 (9折)</t>
+          <t>0.108308 (8.8折)</t>
         </is>
       </c>
       <c r="H47" s="14" t="inlineStr">
         <is>
+          <t>0.270769 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
+        <is>
           <t>0.104615 (8.5折)</t>
         </is>
       </c>
-      <c r="I47" s="14" t="inlineStr">
+      <c r="J47" s="14" t="inlineStr">
         <is>
           <t>0.261538 (8.5折)</t>
         </is>
       </c>
-      <c r="J47" s="14" t="inlineStr">
+      <c r="K47" s="14" t="inlineStr">
         <is>
           <t>0.100923 (8.2折)</t>
         </is>
       </c>
-      <c r="K47" s="14" t="inlineStr">
+      <c r="L47" s="14" t="inlineStr">
         <is>
           <t>0.252307 (8.2折)</t>
         </is>
       </c>
-      <c r="L47" s="14" t="inlineStr">
+      <c r="M47" s="14" t="inlineStr">
         <is>
           <t>0.093539 (7.6折)</t>
         </is>
       </c>
-      <c r="M47" s="14" t="inlineStr">
+      <c r="N47" s="14" t="inlineStr">
         <is>
           <t>0.233846 (7.6折)</t>
         </is>
       </c>
-      <c r="N47" s="14" t="inlineStr">
+      <c r="O47" s="14" t="inlineStr">
         <is>
           <t>0.088615 (7.2折)</t>
         </is>
       </c>
-      <c r="O47" s="14" t="inlineStr">
+      <c r="P47" s="14" t="inlineStr">
         <is>
           <t>0.221538 (7.2折)</t>
         </is>
@@ -4031,50 +4260,55 @@
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
-          <t>0.041539 (9折)</t>
+          <t>0.010345</t>
         </is>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>0.083077 (9折)</t>
+          <t>0.040616 (8.8折)</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
+          <t>0.081231 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
           <t>0.039231 (8.5折)</t>
         </is>
       </c>
-      <c r="I48" s="11" t="inlineStr">
+      <c r="J48" s="11" t="inlineStr">
         <is>
           <t>0.078462 (8.5折)</t>
         </is>
       </c>
-      <c r="J48" s="11" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>0.037846 (8.2折)</t>
         </is>
       </c>
-      <c r="K48" s="11" t="inlineStr">
+      <c r="L48" s="11" t="inlineStr">
         <is>
           <t>0.075693 (8.2折)</t>
         </is>
       </c>
-      <c r="L48" s="11" t="inlineStr">
+      <c r="M48" s="11" t="inlineStr">
         <is>
           <t>0.035077 (7.6折)</t>
         </is>
       </c>
-      <c r="M48" s="11" t="inlineStr">
+      <c r="N48" s="11" t="inlineStr">
         <is>
           <t>0.070154 (7.6折)</t>
         </is>
       </c>
-      <c r="N48" s="11" t="inlineStr">
+      <c r="O48" s="11" t="inlineStr">
         <is>
           <t>0.033231 (7.2折)</t>
         </is>
       </c>
-      <c r="O48" s="11" t="inlineStr">
+      <c r="P48" s="11" t="inlineStr">
         <is>
           <t>0.066462 (7.2折)</t>
         </is>
@@ -4104,50 +4338,55 @@
       </c>
       <c r="F49" s="14" t="inlineStr">
         <is>
-          <t>0.027692 (9折)</t>
+          <t>0.003077</t>
         </is>
       </c>
       <c r="G49" s="14" t="inlineStr">
         <is>
-          <t>0.276923 (9折)</t>
+          <t>0.027077 (8.8折)</t>
         </is>
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
+          <t>0.270769 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr">
+        <is>
           <t>0.026154 (8.5折)</t>
         </is>
       </c>
-      <c r="I49" s="14" t="inlineStr">
+      <c r="J49" s="14" t="inlineStr">
         <is>
           <t>0.261538 (8.5折)</t>
         </is>
       </c>
-      <c r="J49" s="14" t="inlineStr">
+      <c r="K49" s="14" t="inlineStr">
         <is>
           <t>0.025231 (8.2折)</t>
         </is>
       </c>
-      <c r="K49" s="14" t="inlineStr">
+      <c r="L49" s="14" t="inlineStr">
         <is>
           <t>0.252307 (8.2折)</t>
         </is>
       </c>
-      <c r="L49" s="14" t="inlineStr">
+      <c r="M49" s="14" t="inlineStr">
         <is>
           <t>0.023384 (7.6折)</t>
         </is>
       </c>
-      <c r="M49" s="14" t="inlineStr">
+      <c r="N49" s="14" t="inlineStr">
         <is>
           <t>0.233846 (7.6折)</t>
         </is>
       </c>
-      <c r="N49" s="14" t="inlineStr">
+      <c r="O49" s="14" t="inlineStr">
         <is>
           <t>0.022154 (7.2折)</t>
         </is>
       </c>
-      <c r="O49" s="14" t="inlineStr">
+      <c r="P49" s="14" t="inlineStr">
         <is>
           <t>0.221538 (7.2折)</t>
         </is>
@@ -4177,50 +4416,55 @@
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
-          <t>0.110769 (9折)</t>
+          <t>0.012308</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>0.664616 (9折)</t>
+          <t>0.108308 (8.8折)</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
+          <t>0.649847 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
           <t>0.104615 (8.5折)</t>
         </is>
       </c>
-      <c r="I50" s="11" t="inlineStr">
+      <c r="J50" s="11" t="inlineStr">
         <is>
           <t>0.627693 (8.5折)</t>
         </is>
       </c>
-      <c r="J50" s="11" t="inlineStr">
+      <c r="K50" s="11" t="inlineStr">
         <is>
           <t>0.100923 (8.2折)</t>
         </is>
       </c>
-      <c r="K50" s="11" t="inlineStr">
+      <c r="L50" s="11" t="inlineStr">
         <is>
           <t>0.605539 (8.2折)</t>
         </is>
       </c>
-      <c r="L50" s="11" t="inlineStr">
+      <c r="M50" s="11" t="inlineStr">
         <is>
           <t>0.093539 (7.6折)</t>
         </is>
       </c>
-      <c r="M50" s="11" t="inlineStr">
+      <c r="N50" s="11" t="inlineStr">
         <is>
           <t>0.561231 (7.6折)</t>
         </is>
       </c>
-      <c r="N50" s="11" t="inlineStr">
+      <c r="O50" s="11" t="inlineStr">
         <is>
           <t>0.088615 (7.2折)</t>
         </is>
       </c>
-      <c r="O50" s="11" t="inlineStr">
+      <c r="P50" s="11" t="inlineStr">
         <is>
           <t>0.531693 (7.2折)</t>
         </is>
@@ -4250,50 +4494,55 @@
       </c>
       <c r="F51" s="14" t="inlineStr">
         <is>
-          <t>0.166154 (9折)</t>
+          <t>0.036923</t>
         </is>
       </c>
       <c r="G51" s="14" t="inlineStr">
         <is>
-          <t>0.996923 (9折)</t>
+          <t>0.162461 (8.8折)</t>
         </is>
       </c>
       <c r="H51" s="14" t="inlineStr">
         <is>
+          <t>0.974769 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
           <t>0.156923 (8.5折)</t>
         </is>
       </c>
-      <c r="I51" s="14" t="inlineStr">
+      <c r="J51" s="14" t="inlineStr">
         <is>
           <t>0.941538 (8.5折)</t>
         </is>
       </c>
-      <c r="J51" s="14" t="inlineStr">
+      <c r="K51" s="14" t="inlineStr">
         <is>
           <t>0.151384 (8.2折)</t>
         </is>
       </c>
-      <c r="K51" s="14" t="inlineStr">
+      <c r="L51" s="14" t="inlineStr">
         <is>
           <t>0.908307 (8.2折)</t>
         </is>
       </c>
-      <c r="L51" s="14" t="inlineStr">
+      <c r="M51" s="14" t="inlineStr">
         <is>
           <t>0.140307 (7.6折)</t>
         </is>
       </c>
-      <c r="M51" s="14" t="inlineStr">
+      <c r="N51" s="14" t="inlineStr">
         <is>
           <t>0.841846 (7.6折)</t>
         </is>
       </c>
-      <c r="N51" s="14" t="inlineStr">
+      <c r="O51" s="14" t="inlineStr">
         <is>
           <t>0.132923 (7.2折)</t>
         </is>
       </c>
-      <c r="O51" s="14" t="inlineStr">
+      <c r="P51" s="14" t="inlineStr">
         <is>
           <t>0.797538 (7.2折)</t>
         </is>
@@ -4323,50 +4572,55 @@
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>0.276923 (9折)</t>
+          <t>0.061538</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>1.661539 (9折)</t>
+          <t>0.270769 (8.8折)</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
+          <t>1.624616 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
           <t>0.261538 (8.5折)</t>
         </is>
       </c>
-      <c r="I52" s="11" t="inlineStr">
+      <c r="J52" s="11" t="inlineStr">
         <is>
           <t>1.569231 (8.5折)</t>
         </is>
       </c>
-      <c r="J52" s="11" t="inlineStr">
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>0.252307 (8.2折)</t>
         </is>
       </c>
-      <c r="K52" s="11" t="inlineStr">
+      <c r="L52" s="11" t="inlineStr">
         <is>
           <t>1.513846 (8.2折)</t>
         </is>
       </c>
-      <c r="L52" s="11" t="inlineStr">
+      <c r="M52" s="11" t="inlineStr">
         <is>
           <t>0.233846 (7.6折)</t>
         </is>
       </c>
-      <c r="M52" s="11" t="inlineStr">
+      <c r="N52" s="11" t="inlineStr">
         <is>
           <t>1.403077 (7.6折)</t>
         </is>
       </c>
-      <c r="N52" s="11" t="inlineStr">
+      <c r="O52" s="11" t="inlineStr">
         <is>
           <t>0.221538 (7.2折)</t>
         </is>
       </c>
-      <c r="O52" s="11" t="inlineStr">
+      <c r="P52" s="11" t="inlineStr">
         <is>
           <t>1.329231 (7.2折)</t>
         </is>
@@ -4396,50 +4650,55 @@
       </c>
       <c r="F53" s="14" t="inlineStr">
         <is>
-          <t>1.661539 (9折)</t>
+          <t>0.369231</t>
         </is>
       </c>
       <c r="G53" s="14" t="inlineStr">
         <is>
-          <t>4.984616 (9折)</t>
+          <t>1.624616 (8.8折)</t>
         </is>
       </c>
       <c r="H53" s="14" t="inlineStr">
         <is>
+          <t>4.873847 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
           <t>1.569231 (8.5折)</t>
         </is>
       </c>
-      <c r="I53" s="14" t="inlineStr">
+      <c r="J53" s="14" t="inlineStr">
         <is>
           <t>4.707693 (8.5折)</t>
         </is>
       </c>
-      <c r="J53" s="14" t="inlineStr">
+      <c r="K53" s="14" t="inlineStr">
         <is>
           <t>1.513846 (8.2折)</t>
         </is>
       </c>
-      <c r="K53" s="14" t="inlineStr">
+      <c r="L53" s="14" t="inlineStr">
         <is>
           <t>4.541539 (8.2折)</t>
         </is>
       </c>
-      <c r="L53" s="14" t="inlineStr">
+      <c r="M53" s="14" t="inlineStr">
         <is>
           <t>1.403077 (7.6折)</t>
         </is>
       </c>
-      <c r="M53" s="14" t="inlineStr">
+      <c r="N53" s="14" t="inlineStr">
         <is>
           <t>4.209231 (7.6折)</t>
         </is>
       </c>
-      <c r="N53" s="14" t="inlineStr">
+      <c r="O53" s="14" t="inlineStr">
         <is>
           <t>1.329231 (7.2折)</t>
         </is>
       </c>
-      <c r="O53" s="14" t="inlineStr">
+      <c r="P53" s="14" t="inlineStr">
         <is>
           <t>3.987693 (7.2折)</t>
         </is>
@@ -4469,50 +4728,55 @@
       </c>
       <c r="F54" s="11" t="inlineStr">
         <is>
-          <t>0.276923 (9折)</t>
+          <t>0.061538</t>
         </is>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>1.107692 (9折)</t>
+          <t>0.270769 (8.8折)</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
+          <t>1.083077 (8.8折)</t>
+        </is>
+      </c>
+      <c r="I54" s="11" t="inlineStr">
+        <is>
           <t>0.261538 (8.5折)</t>
         </is>
       </c>
-      <c r="I54" s="11" t="inlineStr">
+      <c r="J54" s="11" t="inlineStr">
         <is>
           <t>1.046154 (8.5折)</t>
         </is>
       </c>
-      <c r="J54" s="11" t="inlineStr">
+      <c r="K54" s="11" t="inlineStr">
         <is>
           <t>0.252307 (8.2折)</t>
         </is>
       </c>
-      <c r="K54" s="11" t="inlineStr">
+      <c r="L54" s="11" t="inlineStr">
         <is>
           <t>1.009231 (8.2折)</t>
         </is>
       </c>
-      <c r="L54" s="11" t="inlineStr">
+      <c r="M54" s="11" t="inlineStr">
         <is>
           <t>0.233846 (7.6折)</t>
         </is>
       </c>
-      <c r="M54" s="11" t="inlineStr">
+      <c r="N54" s="11" t="inlineStr">
         <is>
           <t>0.935384 (7.6折)</t>
         </is>
       </c>
-      <c r="N54" s="11" t="inlineStr">
+      <c r="O54" s="11" t="inlineStr">
         <is>
           <t>0.221538 (7.2折)</t>
         </is>
       </c>
-      <c r="O54" s="11" t="inlineStr">
+      <c r="P54" s="11" t="inlineStr">
         <is>
           <t>0.886154 (7.2折)</t>
         </is>
@@ -4551,47 +4815,52 @@
       </c>
       <c r="G55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="H55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="I55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="L55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="M55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="N55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="O55" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
+        </is>
+      </c>
+      <c r="P55" s="14" t="inlineStr">
+        <is>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
     </row>
@@ -4624,47 +4893,52 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.046154 (原价)</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.046154 (原价)</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.046154 (原价)</t>
         </is>
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="M56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.046154 (原价)</t>
         </is>
       </c>
       <c r="N56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="O56" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.046154 (原价)</t>
+        </is>
+      </c>
+      <c r="P56" s="11" t="inlineStr">
+        <is>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
     </row>
@@ -4697,47 +4971,52 @@
       </c>
       <c r="G57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="I57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="L57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="M57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="N57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="O57" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
+        </is>
+      </c>
+      <c r="P57" s="14" t="inlineStr">
+        <is>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
     </row>
@@ -4770,47 +5049,52 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="J58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="M58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
         </is>
       </c>
       <c r="N58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
       <c r="O58" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.076923 (原价)</t>
+        </is>
+      </c>
+      <c r="P58" s="11" t="inlineStr">
+        <is>
+          <t>0.307692 (原价)</t>
         </is>
       </c>
     </row>
@@ -4843,47 +5127,52 @@
       </c>
       <c r="G59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="I59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="K59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="L59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="M59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
         </is>
       </c>
       <c r="N59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
       <c r="O59" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.369231 (原价)</t>
+        </is>
+      </c>
+      <c r="P59" s="14" t="inlineStr">
+        <is>
+          <t>1.476923 (原价)</t>
         </is>
       </c>
     </row>
@@ -4916,47 +5205,52 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.153846 (原价)</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.692308 (原价)</t>
         </is>
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.153846 (原价)</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.692308 (原价)</t>
         </is>
       </c>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.153846 (原价)</t>
         </is>
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.692308 (原价)</t>
         </is>
       </c>
       <c r="M60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.153846 (原价)</t>
         </is>
       </c>
       <c r="N60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.692308 (原价)</t>
         </is>
       </c>
       <c r="O60" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.153846 (原价)</t>
+        </is>
+      </c>
+      <c r="P60" s="11" t="inlineStr">
+        <is>
+          <t>2.692308 (原价)</t>
         </is>
       </c>
     </row>
@@ -4984,77 +5278,83 @@
       </c>
       <c r="F61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.061538</t>
         </is>
       </c>
       <c r="G61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.615385 (原价)</t>
         </is>
       </c>
       <c r="I61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.615385 (原价)</t>
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="L61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.615385 (原价)</t>
         </is>
       </c>
       <c r="M61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.184615 (原价)</t>
         </is>
       </c>
       <c r="N61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.615385 (原价)</t>
         </is>
       </c>
       <c r="O61" s="14" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="72" customHeight="1">
+          <t>0.184615 (原价)</t>
+        </is>
+      </c>
+      <c r="P61" s="14" t="inlineStr">
+        <is>
+          <t>0.615385 (原价)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="78" customHeight="1">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>说明：① 目录价 = 平台标准档刊例；阶梯格 = 目录价 × 对客折（括号内为折数，原价=不打折）。② 达档按商务表：企业户月消耗目录价金额；开通与合同以商务确认为准。③ 交叉模型按「02 推荐成本折」取阶梯；未进商务清单的模型阶梯为「—」，请询价。④ 不含缓存价、成本折、线路与二转；生图/视频另表。⑤ 正式外发前请运营/商务复核。</t>
+          <t>说明：① 目录价 = 平台标准档刊例（输入/输出/缓存；无缓存刊例为「—」）；阶梯格 = 目录入/出价 × 对客折（括号内为折数，原价=不打折）；阶梯暂不含缓存列。② 达档按商务表：企业户月消耗目录价金额；开通与合同以商务确认为准。③ 阶梯按定价方案-v0 公开定折（成本族 0.65/0.70/0.75 + 0.78浅折 + Claude 对齐）；1.0 原价族及未映射模型阶梯写「数字 (原价)」，不用「—」。④ 不含成本折、线路与二转；0.75 族可能含备选线路，公开价仍按上表。⑤ 正式外发前请运营/商务复核。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="J4:K4"/>
+  <mergeCells count="14">
+    <mergeCell ref="A63:P63"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="L4:M4"/>
     <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A1:P1"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A63:O63"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5073,7 +5373,7 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5106,7 +5406,7 @@
       </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
-          <t>阶梯来源</t>
+          <t>公开阶梯来源</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5431,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5456,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5481,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5201,14 +5501,12 @@
           <t>GPT-5 Nano</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D7" t="n">
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>单模对齐0.65公开阶梯（01归属）</t>
         </is>
       </c>
     </row>
@@ -5233,7 +5531,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5556,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5581,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.65（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5308,7 +5606,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.65（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5631,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.65（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5656,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5681,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>0.78浅折→原价档外浅折（01归属）</t>
         </is>
       </c>
     </row>
@@ -5408,7 +5706,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>0.78浅折→原价档外浅折（01归属）</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5731,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>Claude对齐opus阶梯（01归属）</t>
         </is>
       </c>
     </row>
@@ -5458,7 +5756,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>Claude对齐opus阶梯（01归属）</t>
         </is>
       </c>
     </row>
@@ -5483,7 +5781,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>Claude对齐opus阶梯（01归属）</t>
         </is>
       </c>
     </row>
@@ -5508,7 +5806,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>Claude对齐opus阶梯（01归属）</t>
         </is>
       </c>
     </row>
@@ -5533,7 +5831,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5856,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5881,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.75（01归属）</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5906,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5931,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5658,7 +5956,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5981,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5708,7 +6006,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>02 推荐</t>
+          <t>公开族 0.7（02推荐）</t>
         </is>
       </c>
     </row>
@@ -5733,7 +6031,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -5758,7 +6056,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -5778,14 +6076,12 @@
           <t>DeepSeek V4 Pro Direct</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D30" t="n">
+        <v>1</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -5810,7 +6106,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -5835,7 +6131,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -5860,7 +6156,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -5880,14 +6176,12 @@
           <t>Kimi K2.7 Code HighSpeed</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D34" t="n">
+        <v>1</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -5907,14 +6201,12 @@
           <t>MiniMax M2.5</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D35" t="n">
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -5934,14 +6226,12 @@
           <t>MiniMax M2.7</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D36" t="n">
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -5961,14 +6251,12 @@
           <t>MiniMax M3</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D37" t="n">
+        <v>1</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -5993,7 +6281,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -6013,14 +6301,12 @@
           <t>GLM 5 Turbo</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D39" t="n">
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6331,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6356,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.7（01归属）</t>
         </is>
       </c>
     </row>
@@ -6090,14 +6376,12 @@
           <t>GLM-5V Turbo</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D42" t="n">
+        <v>1</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6406,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6431,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6172,7 +6456,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6481,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6506,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6531,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6272,7 +6556,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6297,7 +6581,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6606,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6631,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>01 归属</t>
+          <t>公开族 0.65（01归属）</t>
         </is>
       </c>
     </row>
@@ -6367,14 +6651,12 @@
           <t>Hy-Role Latest</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D53" t="n">
+        <v>1</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6394,14 +6676,12 @@
           <t>Hy-MT2 Lite</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D54" t="n">
+        <v>1</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6421,14 +6701,12 @@
           <t>Hy-MT2 Plus</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D55" t="n">
+        <v>1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6448,14 +6726,12 @@
           <t>Hy-MT2 Pro</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D56" t="n">
+        <v>1</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6475,14 +6751,12 @@
           <t>Hy-Role</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D57" t="n">
+        <v>1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6502,14 +6776,12 @@
           <t>Hy-Vision 2.0 Instruct</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D58" t="n">
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>
@@ -6529,14 +6801,12 @@
           <t>Hy3 Preview</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D59" t="n">
+        <v>1</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>未映射</t>
+          <t>1.0→原价（01归属）</t>
         </is>
       </c>
     </row>

</xml_diff>